<commit_message>
Rebuild Home Command Center marketing as dense, authentic app screenshots
Replace the sparse mockups with screenshot-style images that mirror the real
workbook: a left sidebar listing all 28 tabs, the REAL computed KPI numbers
from the sample data (budget left $223, bills 8/12, meal plan 91%, home
health 62%, etc.), and fully populated tables — the full 18-row budget with
over-budget data bars, the 12-row bill list with paid/due/overdue pills, the
weekly meal grid, and the cleaning/chore table. Adds an 'Everything Inside —
28 tabs' showcase image. Also marks the auto-pay bills paid in the workbook
so the marketing numbers are truthful to the file.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016YnPMpeJWKT9dx5HR1K2in
</commit_message>
<xml_diff>
--- a/products/home-command-center/Home_Command_Center.xlsx
+++ b/products/home-command-center/Home_Command_Center.xlsx
@@ -17890,10 +17890,14 @@
       </c>
       <c r="F5" s="17" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G5" s="16" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G5" s="16" t="inlineStr">
+        <is>
+          <t>CONF-10231</t>
+        </is>
+      </c>
       <c r="H5" s="18" t="n">
         <v>46538</v>
       </c>
@@ -17931,10 +17935,14 @@
       </c>
       <c r="F6" s="20" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G6" s="19" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G6" s="19" t="inlineStr">
+        <is>
+          <t>CONF-44120</t>
+        </is>
+      </c>
       <c r="H6" s="21" t="inlineStr"/>
       <c r="J6" s="27" t="inlineStr">
         <is>
@@ -18000,10 +18008,14 @@
       </c>
       <c r="F8" s="20" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G8" s="19" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G8" s="19" t="inlineStr">
+        <is>
+          <t>CONF-90021</t>
+        </is>
+      </c>
       <c r="H8" s="21" t="inlineStr"/>
       <c r="J8" s="23" t="inlineStr">
         <is>
@@ -18039,10 +18051,14 @@
       </c>
       <c r="F9" s="17" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G9" s="16" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G9" s="16" t="inlineStr">
+        <is>
+          <t>CONF-77410</t>
+        </is>
+      </c>
       <c r="H9" s="18" t="inlineStr"/>
     </row>
     <row r="10">
@@ -18069,10 +18085,14 @@
       </c>
       <c r="F10" s="20" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G10" s="19" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G10" s="19" t="inlineStr">
+        <is>
+          <t>CONF-22018</t>
+        </is>
+      </c>
       <c r="H10" s="21" t="n">
         <v>46323</v>
       </c>
@@ -18101,10 +18121,14 @@
       </c>
       <c r="F11" s="17" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G11" s="16" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G11" s="16" t="inlineStr">
+        <is>
+          <t>CONF-22019</t>
+        </is>
+      </c>
       <c r="H11" s="18" t="n">
         <v>46298</v>
       </c>

</xml_diff>